<commit_message>
medication separated for tablets, patches, liquids!
</commit_message>
<xml_diff>
--- a/inst/extdata/Med_calc.xlsx
+++ b/inst/extdata/Med_calc.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sheej\Documents\Sheeja_WinLap\repos\packDAMipd\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{967AC4D9-3E26-4CF4-B4CC-C22FC2A2CF64}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD60E52E-E7AB-4CF7-A85C-B03A6D8DB0EA}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="38">
   <si>
     <t>Morphine</t>
   </si>
@@ -144,6 +144,9 @@
   </si>
   <si>
     <t>patches</t>
+  </si>
+  <si>
+    <t xml:space="preserve">it shold be 1 </t>
   </si>
 </sst>
 </file>
@@ -747,7 +750,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -761,7 +764,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>18</v>
       </c>
@@ -775,7 +778,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -789,7 +792,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -803,7 +806,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>16</v>
       </c>
@@ -817,7 +820,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>15</v>
       </c>
@@ -831,7 +834,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>0</v>
       </c>
@@ -841,11 +844,14 @@
       <c r="C23" t="s">
         <v>14</v>
       </c>
-      <c r="D23">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D23" t="s">
+        <v>4</v>
+      </c>
+      <c r="E23" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
meducations costing long dara fornat
</commit_message>
<xml_diff>
--- a/inst/extdata/Med_calc.xlsx
+++ b/inst/extdata/Med_calc.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sheej\Documents\Sheeja_WinLap\repos\packDAMipd\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD60E52E-E7AB-4CF7-A85C-B03A6D8DB0EA}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7084FCEB-83BD-4AE9-908E-6EEA9F58FC58}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="37">
   <si>
     <t>Morphine</t>
   </si>
@@ -144,9 +144,6 @@
   </si>
   <si>
     <t>patches</t>
-  </si>
-  <si>
-    <t xml:space="preserve">it shold be 1 </t>
   </si>
 </sst>
 </file>
@@ -750,7 +747,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -764,7 +761,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>18</v>
       </c>
@@ -778,7 +775,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -792,7 +789,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -806,7 +803,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>16</v>
       </c>
@@ -820,7 +817,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>15</v>
       </c>
@@ -834,7 +831,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>0</v>
       </c>
@@ -845,13 +842,10 @@
         <v>14</v>
       </c>
       <c r="D23" t="s">
-        <v>4</v>
-      </c>
-      <c r="E23" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
modified cost medication function
</commit_message>
<xml_diff>
--- a/inst/extdata/Med_calc.xlsx
+++ b/inst/extdata/Med_calc.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23127"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sheej\Documents\Sheeja_WinLap\repos\packDAMipd\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7084FCEB-83BD-4AE9-908E-6EEA9F58FC58}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2657D223-4A92-4CC2-B1DC-80C49CC5CBA6}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="38">
   <si>
     <t>Morphine</t>
   </si>
@@ -144,6 +144,9 @@
   </si>
   <si>
     <t>patches</t>
+  </si>
+  <si>
+    <t>Others</t>
   </si>
 </sst>
 </file>
@@ -513,7 +516,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.7109375" customWidth="1"/>
@@ -859,6 +862,14 @@
         <v>1.5</v>
       </c>
     </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>37</v>
+      </c>
+      <c r="D25">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
MED calc table corrected
</commit_message>
<xml_diff>
--- a/inst/extdata/Med_calc.xlsx
+++ b/inst/extdata/Med_calc.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sheej\Documents\Sheeja_WinLap\repos\packDAMipd\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16ADA9B8-ED98-417A-B21E-807102528C12}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A681BBF-D1E2-462B-9A73-F0733F741E66}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="840" yWindow="315" windowWidth="19545" windowHeight="8520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="KB" sheetId="2" r:id="rId1"/>
@@ -595,13 +595,10 @@
         <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="D5">
         <v>0.15</v>
-      </c>
-      <c r="E5" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -612,10 +609,13 @@
         <v>9</v>
       </c>
       <c r="C6" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D6">
         <v>0.1</v>
+      </c>
+      <c r="E6" t="s">
+        <v>22</v>
       </c>
       <c r="H6" s="1"/>
     </row>

</xml_diff>

<commit_message>
tablets- added NA dose and mix drug
</commit_message>
<xml_diff>
--- a/inst/extdata/Med_calc.xlsx
+++ b/inst/extdata/Med_calc.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23901"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sheej\Documents\Sheeja_WinLap\repos\packDAMipd\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A681BBF-D1E2-462B-9A73-F0733F741E66}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B081DA94-E6DB-4909-97ED-C977FD86C729}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -68,18 +68,6 @@
     <t>mg</t>
   </si>
   <si>
-    <t>8/500 mg</t>
-  </si>
-  <si>
-    <t>15/500 mg</t>
-  </si>
-  <si>
-    <t>30/500 mg</t>
-  </si>
-  <si>
-    <t>10/500 mg</t>
-  </si>
-  <si>
     <t>patch</t>
   </si>
   <si>
@@ -147,6 +135,18 @@
   </si>
   <si>
     <t>Others</t>
+  </si>
+  <si>
+    <t>8mg/500mg</t>
+  </si>
+  <si>
+    <t>15mg/500mg</t>
+  </si>
+  <si>
+    <t>10mg/500mg</t>
+  </si>
+  <si>
+    <t>30mg/500mg</t>
   </si>
 </sst>
 </file>
@@ -530,21 +530,21 @@
         <v>5</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
         <v>7</v>
@@ -558,7 +558,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>
@@ -572,7 +572,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B4" t="s">
         <v>9</v>
@@ -584,12 +584,12 @@
         <v>0.15</v>
       </c>
       <c r="E4" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
@@ -603,7 +603,7 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B6" t="s">
         <v>9</v>
@@ -615,7 +615,7 @@
         <v>0.1</v>
       </c>
       <c r="E6" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="H6" s="1"/>
     </row>
@@ -635,7 +635,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B8" t="s">
         <v>9</v>
@@ -649,7 +649,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B9" t="s">
         <v>9</v>
@@ -663,7 +663,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B10" t="s">
         <v>9</v>
@@ -705,7 +705,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B13" t="s">
         <v>9</v>
@@ -719,7 +719,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B14" t="s">
         <v>9</v>
@@ -733,7 +733,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B15" t="s">
         <v>9</v>
@@ -747,7 +747,7 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B16" t="s">
         <v>9</v>
@@ -761,13 +761,13 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B17" t="s">
         <v>9</v>
       </c>
       <c r="C17" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="D17">
         <v>0.15</v>
@@ -775,13 +775,13 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B18" t="s">
         <v>9</v>
       </c>
       <c r="C18" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="D18">
         <v>0.15</v>
@@ -789,13 +789,13 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B19" t="s">
         <v>9</v>
       </c>
       <c r="C19" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="D19">
         <v>0.15</v>
@@ -803,13 +803,13 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B20" t="s">
         <v>9</v>
       </c>
       <c r="C20" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="D20">
         <v>0.1</v>
@@ -817,13 +817,13 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B21" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C21" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D21" t="s">
         <v>4</v>
@@ -831,13 +831,13 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C22" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D22" t="s">
         <v>4</v>
@@ -848,10 +848,10 @@
         <v>1</v>
       </c>
       <c r="B23" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C23" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D23">
         <v>1</v>
@@ -862,10 +862,10 @@
         <v>2</v>
       </c>
       <c r="B24" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C24" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D24">
         <v>1.5</v>
@@ -873,7 +873,7 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="D25">
         <v>0</v>

</xml_diff>